<commit_message>
feat: add enable_ai_insights to config template; regenerate xlsx
Adds AI INSIGHTS section to the Settings sheet with enable_ai_insights
field (default FALSE, dropdown TRUE/FALSE). Includes description noting
the ANTHROPIC_API_KEY requirement.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/tabs/templates/Crosstab_Config_Template.xlsx
+++ b/modules/tabs/templates/Crosstab_Config_Template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="369">
   <si>
     <t xml:space="preserve">TURAS Crosstab Configuration</t>
   </si>
@@ -832,6 +832,15 @@
   </si>
   <si>
     <t xml:space="preserve">Y or N (see description)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI INSIGHTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable_ai_insights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate AI-powered callout insights alongside crosstab tables in the HTML report. Requires an Anthropic API key set in the ANTHROPIC_API_KEY environment variable. Leave FALSE if you do not have an API key or do not need AI commentary.</t>
   </si>
   <si>
     <t xml:space="preserve">STUDY IDENTIFICATION</t>
@@ -3375,7 +3384,7 @@
         <v>273</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C113" s="16" t="s">
         <v>4</v>
@@ -3384,29 +3393,21 @@
         <v>274</v>
       </c>
       <c r="E113" s="14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="9" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="B114" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C114" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D114" s="13" t="s">
-        <v>277</v>
-      </c>
-      <c r="E114" s="14" t="s">
-        <v>275</v>
-      </c>
+      <c r="B114" s="9"/>
+      <c r="C114" s="9"/>
+      <c r="D114" s="9"/>
+      <c r="E114" s="9"/>
     </row>
     <row r="115">
       <c r="A115" s="15" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B115" s="11" t="s">
         <v>36</v>
@@ -3415,14 +3416,48 @@
         <v>4</v>
       </c>
       <c r="D115" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="E115" s="14" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="E115" s="14" t="s">
-        <v>275</v>
+      <c r="B116" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C116" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D116" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="E116" s="14" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="15" t="s">
+        <v>281</v>
+      </c>
+      <c r="B117" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C117" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D117" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="E117" s="14" t="s">
+        <v>278</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A6:E6"/>
@@ -3441,6 +3476,7 @@
     <mergeCell ref="A100:E100"/>
     <mergeCell ref="A105:E105"/>
     <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A114:E114"/>
   </mergeCells>
   <dataValidations count="20">
     <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B17:B17">
@@ -3528,7 +3564,7 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="37">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="38">
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"xlsx,csv"</xm:f>
@@ -3751,6 +3787,12 @@
           </x14:formula1>
           <xm:sqref>B111:B111</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"FALSE,TRUE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B113:B113</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -3776,99 +3818,99 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>128</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="F5" s="17" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="H5" s="17" t="s">
         <v>36</v>
@@ -3877,30 +3919,30 @@
         <v>36</v>
       </c>
       <c r="J5" s="17" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>128</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>36</v>
@@ -3909,18 +3951,18 @@
         <v>36</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>128</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>36</v>
@@ -3941,7 +3983,7 @@
         <v>36</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8">
@@ -4602,122 +4644,122 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -4742,42 +4784,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>36</v>
@@ -4785,10 +4827,10 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>36</v>
@@ -4796,10 +4838,10 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>36</v>
@@ -4977,42 +5019,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>1</v>
@@ -5020,10 +5062,10 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
docs(tabs): add the data-centric report v2 keys to the config template
The v2 / tracker Settings keys existed in the config parser + whitelist but were
missing from the config template an analyst generates — so they were
undiscoverable. Adds a "DATA-CENTRIC REPORT V2 (OPTIONAL)" section to
generate_config_templates.R (html_report_v2, sampling_method, wave,
html_report_v2_tracking, waves_source, wave_order, question_mapping), regenerates
Crosstab_Config_Template.xlsx, and documents them in 06_TEMPLATE_REFERENCE.md.

Additive + off by default. Template generator tests pass (29/0).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/tabs/templates/Crosstab_Config_Template.xlsx
+++ b/modules/tabs/templates/Crosstab_Config_Template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="393">
   <si>
     <t xml:space="preserve">TURAS Crosstab Configuration</t>
   </si>
@@ -597,12 +597,21 @@
     <t xml:space="preserve">#CC9900</t>
   </si>
   <si>
-    <t xml:space="preserve">Accent colour for HTML report highlights and call-outs.</t>
+    <t xml:space="preserve">Accent colour for HTML report highlights and call-outs. Also used as the default crosstab heatmap tint colour.</t>
   </si>
   <si>
     <t xml:space="preserve">Hex colour code (e.g. #CC9900)</t>
   </si>
   <si>
+    <t xml:space="preserve">heatmap_colour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crosstab heatmap cell tint colour. Defaults to accent_colour (warm cream for standard #CC9900). Set explicitly to override without affecting other colours (e.g. #323367 for cool blue).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hex colour code, or leave blank to use accent_colour</t>
+  </si>
+  <si>
     <t xml:space="preserve">chart_bar_colour</t>
   </si>
   <si>
@@ -745,6 +754,69 @@
   </si>
   <si>
     <t xml:space="preserve">File path (deprecated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATA-CENTRIC REPORT V2 (OPTIONAL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_report_v2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Also build the interactive, self-contained data-centric report v2 (live audience filter, custom banners, confidence intervals). Additive: the classic Excel/HTML outputs are unchanged. See docs/11_DATA_CENTRIC_REPORT_V2.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sampling_method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not_Specified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample design — drives honest confidence vocabulary in the v2 report (probability designs speak confidence intervals / margin of error; otherwise stability intervals / point estimates).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not_Specified, Random, Stratified, Cluster, Census, Convenience, Quota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wave label shown in the v2 report header and used as the tracking trend label (e.g. Wave 25 - May 2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free text, or leave blank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_report_v2_tracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add a Tracking tab to the v2 report, built from anonymised per-wave microdata. Requires html_report_v2=TRUE and a waves_source with prior waves' contributions. The standalone tracker module is unaffected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">waves_source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folder holding prior waves' *_wave.json tracking contributions (each wave's own tabs run writes one). Blank -&gt; no history, Tracking tab stays hidden.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folder path, or leave blank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wave_order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numeric x-axis order key for this wave (e.g. 2025.5 so two same-year waves never collide). Blank -&gt; a 4-digit year is parsed from the wave label.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number (e.g. 2026 or 2025.5), or leave blank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">question_mapping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Path to the classic tracker's Question_Mapping.xlsx. Links waves by a canonical key (robust to question renames) + curates which metrics track. Blank -&gt; auto-detected in waves_source, else metrics match by question title.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">File path, or leave blank to auto-detect</t>
   </si>
   <si>
     <t xml:space="preserve">ROW DESCRIPTORS (HTML Report)</t>
@@ -2894,28 +2966,28 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="10" t="s">
+      <c r="A83" s="15" t="s">
         <v>195</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>188</v>
-      </c>
-      <c r="C83" s="12" t="s">
-        <v>15</v>
+        <v>36</v>
+      </c>
+      <c r="C83" s="16" t="s">
+        <v>4</v>
       </c>
       <c r="D83" s="13" t="s">
         <v>196</v>
       </c>
       <c r="E83" s="14" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="C84" s="12" t="s">
         <v>15</v>
@@ -2924,18 +2996,18 @@
         <v>199</v>
       </c>
       <c r="E84" s="14" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="15" t="s">
+      <c r="B85" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="B85" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C85" s="16" t="s">
-        <v>4</v>
+      <c r="C85" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="D85" s="13" t="s">
         <v>202</v>
@@ -3064,76 +3136,76 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="10" t="s">
+      <c r="A93" s="15" t="s">
         <v>225</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C93" s="12" t="s">
-        <v>15</v>
+        <v>36</v>
+      </c>
+      <c r="C93" s="16" t="s">
+        <v>4</v>
       </c>
       <c r="D93" s="13" t="s">
         <v>226</v>
       </c>
       <c r="E93" s="14" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="B94" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C94" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D94" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="E94" s="14" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="15" t="s">
-        <v>227</v>
-      </c>
-      <c r="B94" s="11" t="s">
+    <row r="95">
+      <c r="A95" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="B95" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C94" s="16" t="s">
+      <c r="C95" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D94" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="E94" s="14" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="B95" s="11" t="s">
+      <c r="D95" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="C95" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D95" s="13" t="s">
+      <c r="E95" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="E95" s="14" t="s">
-        <v>229</v>
-      </c>
     </row>
     <row r="96">
-      <c r="A96" s="15" t="s">
+      <c r="A96" s="10" t="s">
         <v>233</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C96" s="16" t="s">
-        <v>4</v>
+        <v>234</v>
+      </c>
+      <c r="C96" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="D96" s="13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E96" s="14" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B97" s="11" t="s">
         <v>36</v>
@@ -3142,10 +3214,10 @@
         <v>4</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E97" s="14" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="98">
@@ -3162,12 +3234,12 @@
         <v>239</v>
       </c>
       <c r="E98" s="14" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="15" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B99" s="11" t="s">
         <v>36</v>
@@ -3176,44 +3248,44 @@
         <v>4</v>
       </c>
       <c r="D99" s="13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E99" s="14" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="9" t="s">
+      <c r="A100" s="15" t="s">
         <v>243</v>
       </c>
-      <c r="B100" s="9"/>
-      <c r="C100" s="9"/>
-      <c r="D100" s="9"/>
-      <c r="E100" s="9"/>
+      <c r="B100" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C100" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D100" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="E100" s="14" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="B101" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C101" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D101" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="E101" s="14" t="s">
+      <c r="A101" s="9" t="s">
         <v>246</v>
       </c>
+      <c r="B101" s="9"/>
+      <c r="C101" s="9"/>
+      <c r="D101" s="9"/>
+      <c r="E101" s="9"/>
     </row>
     <row r="102">
       <c r="A102" s="15" t="s">
         <v>247</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C102" s="16" t="s">
         <v>4</v>
@@ -3222,15 +3294,15 @@
         <v>248</v>
       </c>
       <c r="E102" s="14" t="s">
-        <v>249</v>
+        <v>34</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="B103" s="11" t="s">
         <v>250</v>
-      </c>
-      <c r="B103" s="11" t="s">
-        <v>36</v>
       </c>
       <c r="C103" s="16" t="s">
         <v>4</v>
@@ -3256,21 +3328,29 @@
         <v>254</v>
       </c>
       <c r="E104" s="14" t="s">
-        <v>229</v>
+        <v>255</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="B105" s="9"/>
-      <c r="C105" s="9"/>
-      <c r="D105" s="9"/>
-      <c r="E105" s="9"/>
+      <c r="A105" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="B105" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C105" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D105" s="13" t="s">
+        <v>257</v>
+      </c>
+      <c r="E105" s="14" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="15" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B106" s="11" t="s">
         <v>36</v>
@@ -3279,15 +3359,15 @@
         <v>4</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E106" s="14" t="s">
-        <v>229</v>
+        <v>260</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="15" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B107" s="11" t="s">
         <v>36</v>
@@ -3296,15 +3376,15 @@
         <v>4</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E107" s="14" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="15" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B108" s="11" t="s">
         <v>36</v>
@@ -3313,32 +3393,24 @@
         <v>4</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E108" s="14" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="15" t="s">
-        <v>264</v>
-      </c>
-      <c r="B109" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C109" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D109" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="E109" s="14" t="s">
-        <v>237</v>
-      </c>
+      <c r="A109" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="B109" s="9"/>
+      <c r="C109" s="9"/>
+      <c r="D109" s="9"/>
+      <c r="E109" s="9"/>
     </row>
     <row r="110">
       <c r="A110" s="15" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B110" s="11" t="s">
         <v>36</v>
@@ -3347,58 +3419,66 @@
         <v>4</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E110" s="14" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="15" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B111" s="11" t="s">
-        <v>128</v>
+        <v>36</v>
       </c>
       <c r="C111" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D111" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E111" s="14" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="B112" s="9"/>
-      <c r="C112" s="9"/>
-      <c r="D112" s="9"/>
-      <c r="E112" s="9"/>
+      <c r="A112" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="B112" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C112" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D112" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="E112" s="14" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="15" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C113" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D113" s="13" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="E113" s="14" t="s">
-        <v>34</v>
+        <v>232</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="9" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B114" s="9"/>
       <c r="C114" s="9"/>
@@ -3407,7 +3487,7 @@
     </row>
     <row r="115">
       <c r="A115" s="15" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B115" s="11" t="s">
         <v>36</v>
@@ -3416,15 +3496,15 @@
         <v>4</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="E115" s="14" t="s">
-        <v>278</v>
+        <v>232</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="15" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B116" s="11" t="s">
         <v>36</v>
@@ -3433,15 +3513,15 @@
         <v>4</v>
       </c>
       <c r="D116" s="13" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E116" s="14" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="15" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B117" s="11" t="s">
         <v>36</v>
@@ -3450,14 +3530,151 @@
         <v>4</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E117" s="14" t="s">
-        <v>278</v>
+        <v>287</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="B118" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C118" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D118" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="E118" s="14" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="B119" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C119" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D119" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="E119" s="14" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="15" t="s">
+        <v>293</v>
+      </c>
+      <c r="B120" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="C120" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D120" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="E120" s="14" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="B121" s="9"/>
+      <c r="C121" s="9"/>
+      <c r="D121" s="9"/>
+      <c r="E121" s="9"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="15" t="s">
+        <v>297</v>
+      </c>
+      <c r="B122" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C122" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D122" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="E122" s="14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="B123" s="9"/>
+      <c r="C123" s="9"/>
+      <c r="D123" s="9"/>
+      <c r="E123" s="9"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="B124" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C124" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D124" s="13" t="s">
+        <v>301</v>
+      </c>
+      <c r="E124" s="14" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="15" t="s">
+        <v>303</v>
+      </c>
+      <c r="B125" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C125" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D125" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="E125" s="14" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="B126" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C126" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D126" s="13" t="s">
+        <v>306</v>
+      </c>
+      <c r="E126" s="14" t="s">
+        <v>302</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A6:E6"/>
@@ -3473,10 +3690,11 @@
     <mergeCell ref="A63:E63"/>
     <mergeCell ref="A68:E68"/>
     <mergeCell ref="A79:E79"/>
-    <mergeCell ref="A100:E100"/>
-    <mergeCell ref="A105:E105"/>
-    <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A109:E109"/>
     <mergeCell ref="A114:E114"/>
+    <mergeCell ref="A121:E121"/>
+    <mergeCell ref="A123:E123"/>
   </mergeCells>
   <dataValidations count="20">
     <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B17:B17">
@@ -3564,7 +3782,7 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="38">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="41">
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"xlsx,csv"</xm:f>
@@ -3773,25 +3991,43 @@
           <x14:formula1>
             <xm:f>"warm,cool,research,teal,red,brand"</xm:f>
           </x14:formula1>
-          <xm:sqref>B84:B84</xm:sqref>
+          <xm:sqref>B85:B85</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B93:B93</xm:sqref>
+          <xm:sqref>B94:B94</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B102:B102</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Not_Specified,Random,Stratified,Cluster,Census,Convenience,Quota"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B103:B103</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B105:B105</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"Y,N"</xm:f>
           </x14:formula1>
-          <xm:sqref>B111:B111</xm:sqref>
+          <xm:sqref>B120:B120</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"FALSE,TRUE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B113:B113</xm:sqref>
+          <xm:sqref>B122:B122</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3818,99 +4054,99 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>283</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>284</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>285</v>
+        <v>309</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>286</v>
+        <v>310</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>287</v>
+        <v>311</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>288</v>
+        <v>312</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>289</v>
+        <v>313</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>290</v>
+        <v>314</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>291</v>
+        <v>315</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>292</v>
+        <v>316</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>293</v>
+        <v>317</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>294</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>295</v>
+        <v>319</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>296</v>
+        <v>320</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>297</v>
+        <v>321</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>298</v>
+        <v>322</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>299</v>
+        <v>323</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>300</v>
+        <v>324</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>301</v>
+        <v>325</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>302</v>
+        <v>326</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>303</v>
+        <v>327</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>304</v>
+        <v>328</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>305</v>
+        <v>329</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>128</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>305</v>
+        <v>329</v>
       </c>
       <c r="F5" s="17" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="H5" s="17" t="s">
         <v>36</v>
@@ -3919,30 +4155,30 @@
         <v>36</v>
       </c>
       <c r="J5" s="17" t="s">
-        <v>307</v>
+        <v>331</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>308</v>
+        <v>332</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>128</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>309</v>
+        <v>333</v>
       </c>
       <c r="F6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>36</v>
@@ -3951,18 +4187,18 @@
         <v>36</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>310</v>
+        <v>334</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>311</v>
+        <v>335</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>128</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>36</v>
@@ -3983,7 +4219,7 @@
         <v>36</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>312</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8">
@@ -4644,122 +4880,122 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>313</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>314</v>
+        <v>338</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>315</v>
+        <v>339</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>316</v>
+        <v>340</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>317</v>
+        <v>341</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="s">
-        <v>318</v>
+        <v>342</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>319</v>
+        <v>343</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>320</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="s">
-        <v>321</v>
+        <v>345</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>322</v>
+        <v>346</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>323</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="s">
-        <v>324</v>
+        <v>348</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>325</v>
+        <v>349</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>326</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="s">
-        <v>327</v>
+        <v>351</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>328</v>
+        <v>352</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>329</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="s">
-        <v>330</v>
+        <v>354</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>331</v>
+        <v>355</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>332</v>
+        <v>356</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="s">
-        <v>333</v>
+        <v>357</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>335</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="s">
-        <v>336</v>
+        <v>360</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>337</v>
+        <v>361</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>338</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="s">
-        <v>339</v>
+        <v>363</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>340</v>
+        <v>364</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>341</v>
+        <v>365</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="s">
-        <v>342</v>
+        <v>366</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>343</v>
+        <v>367</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>344</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>
@@ -4784,42 +5020,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>345</v>
+        <v>369</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>285</v>
+        <v>309</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>347</v>
+        <v>371</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>348</v>
+        <v>372</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>349</v>
+        <v>373</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>350</v>
+        <v>374</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>351</v>
+        <v>375</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>352</v>
+        <v>376</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>353</v>
+        <v>377</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>36</v>
@@ -4827,10 +5063,10 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>354</v>
+        <v>378</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>355</v>
+        <v>379</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>36</v>
@@ -4838,10 +5074,10 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>311</v>
+        <v>335</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>356</v>
+        <v>380</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>36</v>
@@ -5019,42 +5255,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>357</v>
+        <v>381</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>358</v>
+        <v>382</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>359</v>
+        <v>383</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>360</v>
+        <v>384</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>361</v>
+        <v>385</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>362</v>
+        <v>386</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>363</v>
+        <v>387</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>364</v>
+        <v>388</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>365</v>
+        <v>389</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>366</v>
+        <v>390</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>1</v>
@@ -5062,10 +5298,10 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>367</v>
+        <v>391</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>368</v>
+        <v>392</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
chore(tabs): add CommentSheet/CommentLink to the config template (Duncan's hand-fix)
The two open-end link columns, placed left of QuestionText (cols L/M), edited directly in
Excel — the template has an embedded drawing that doesn't survive an openxlsx round-trip.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/tabs/templates/Crosstab_Config_Template.xlsx
+++ b/modules/tabs/templates/Crosstab_Config_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duncan/Dev/Turas/modules/tabs/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A3881B-6F2F-F14E-BD24-7DD1E13E3671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAAA661-30B4-8248-AD87-317274ED18C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="19480" windowHeight="11520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="418">
   <si>
     <t>TURAS Crosstab Configuration</t>
   </si>
@@ -1269,6 +1269,18 @@
   </si>
   <si>
     <t>set the order of the category</t>
+  </si>
+  <si>
+    <t>CommentSheet</t>
+  </si>
+  <si>
+    <t>CommentLink</t>
+  </si>
+  <si>
+    <t>The sheet containing open ended comments</t>
+  </si>
+  <si>
+    <t>The close ended question the comments link to</t>
   </si>
 </sst>
 </file>
@@ -3812,26 +3824,26 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A79:E79"/>
     <mergeCell ref="A101:E101"/>
     <mergeCell ref="A110:E110"/>
     <mergeCell ref="A115:E115"/>
     <mergeCell ref="A122:E122"/>
     <mergeCell ref="A125:E125"/>
-    <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A61:E61"/>
-    <mergeCell ref="A63:E63"/>
-    <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A79:E79"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A20:E20"/>
   </mergeCells>
   <dataValidations count="21">
     <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" sqref="B77:B78 B71:B72 B17:B18" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -3913,7 +3925,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
@@ -3924,11 +3936,11 @@
     <col min="6" max="6" width="14.6640625" customWidth="1"/>
     <col min="7" max="7" width="13.6640625" customWidth="1"/>
     <col min="8" max="8" width="35.6640625" customWidth="1"/>
-    <col min="9" max="11" width="30.6640625" customWidth="1"/>
-    <col min="12" max="12" width="40.6640625" customWidth="1"/>
+    <col min="9" max="13" width="30.6640625" customWidth="1"/>
+    <col min="14" max="14" width="40.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="19" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
         <v>314</v>
       </c>
@@ -3943,8 +3955,10 @@
       <c r="J1" s="16"/>
       <c r="K1" s="16"/>
       <c r="L1" s="16"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>315</v>
       </c>
@@ -3959,8 +3973,10 @@
       <c r="J2" s="16"/>
       <c r="K2" s="16"/>
       <c r="L2" s="16"/>
-    </row>
-    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+    </row>
+    <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>316</v>
       </c>
@@ -3995,10 +4011,16 @@
         <v>411</v>
       </c>
       <c r="L3" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="N3" s="6" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>326</v>
       </c>
@@ -4033,10 +4055,16 @@
         <v>413</v>
       </c>
       <c r="L4" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="N4" s="10" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
         <v>336</v>
       </c>
@@ -4066,11 +4094,13 @@
       </c>
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
-      <c r="L5" s="14" t="s">
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>339</v>
       </c>
@@ -4100,11 +4130,13 @@
       </c>
       <c r="J6" s="14"/>
       <c r="K6" s="14"/>
-      <c r="L6" s="14" t="s">
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>342</v>
       </c>
@@ -4134,11 +4166,13 @@
       </c>
       <c r="J7" s="14"/>
       <c r="K7" s="14"/>
-      <c r="L7" s="14" t="s">
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4151,8 +4185,10 @@
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4165,8 +4201,10 @@
       <c r="J9" s="8"/>
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4179,8 +4217,10 @@
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>
       <c r="L10" s="8"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4193,8 +4233,10 @@
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
       <c r="L11" s="8"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4207,8 +4249,10 @@
       <c r="J12" s="8"/>
       <c r="K12" s="8"/>
       <c r="L12" s="8"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4221,8 +4265,10 @@
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
       <c r="L13" s="8"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4235,8 +4281,10 @@
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
       <c r="L14" s="8"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4249,8 +4297,10 @@
       <c r="J15" s="8"/>
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -4263,8 +4313,10 @@
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -4277,8 +4329,10 @@
       <c r="J17" s="8"/>
       <c r="K17" s="8"/>
       <c r="L17" s="8"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -4291,8 +4345,10 @@
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
       <c r="L18" s="8"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -4305,8 +4361,10 @@
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
       <c r="L19" s="8"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -4319,8 +4377,10 @@
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
       <c r="L20" s="8"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -4333,8 +4393,10 @@
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -4347,8 +4409,10 @@
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -4361,8 +4425,10 @@
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
       <c r="L23" s="8"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -4375,8 +4441,10 @@
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
       <c r="L24" s="8"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -4389,8 +4457,10 @@
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
       <c r="L25" s="8"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -4403,8 +4473,10 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
       <c r="L26" s="8"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -4417,8 +4489,10 @@
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -4431,8 +4505,10 @@
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -4445,8 +4521,10 @@
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
       <c r="L29" s="8"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -4459,8 +4537,10 @@
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
       <c r="L30" s="8"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M30" s="8"/>
+      <c r="N30" s="8"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="8"/>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
@@ -4473,8 +4553,10 @@
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -4487,8 +4569,10 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M32" s="8"/>
+      <c r="N32" s="8"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -4501,8 +4585,10 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -4515,8 +4601,10 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M34" s="8"/>
+      <c r="N34" s="8"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -4529,8 +4617,10 @@
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -4543,8 +4633,10 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
       <c r="L36" s="8"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M36" s="8"/>
+      <c r="N36" s="8"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="8"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -4557,8 +4649,10 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
       <c r="L37" s="8"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M37" s="8"/>
+      <c r="N37" s="8"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="8"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
@@ -4571,8 +4665,10 @@
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
       <c r="L38" s="8"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M38" s="8"/>
+      <c r="N38" s="8"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="8"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -4585,8 +4681,10 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -4599,8 +4697,10 @@
       <c r="J40" s="8"/>
       <c r="K40" s="8"/>
       <c r="L40" s="8"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M40" s="8"/>
+      <c r="N40" s="8"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="8"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -4613,8 +4713,10 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
       <c r="L41" s="8"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M41" s="8"/>
+      <c r="N41" s="8"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -4627,8 +4729,10 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M42" s="8"/>
+      <c r="N42" s="8"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -4641,8 +4745,10 @@
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
       <c r="L43" s="8"/>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M43" s="8"/>
+      <c r="N43" s="8"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="8"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -4655,8 +4761,10 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
       <c r="L44" s="8"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M44" s="8"/>
+      <c r="N44" s="8"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="8"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -4669,8 +4777,10 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
       <c r="L45" s="8"/>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M45" s="8"/>
+      <c r="N45" s="8"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -4683,8 +4793,10 @@
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
       <c r="L46" s="8"/>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M46" s="8"/>
+      <c r="N46" s="8"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -4697,8 +4809,10 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
       <c r="L47" s="8"/>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M47" s="8"/>
+      <c r="N47" s="8"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -4711,8 +4825,10 @@
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
       <c r="L48" s="8"/>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M48" s="8"/>
+      <c r="N48" s="8"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="8"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -4725,8 +4841,10 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
       <c r="L49" s="8"/>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M49" s="8"/>
+      <c r="N49" s="8"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="8"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -4739,8 +4857,10 @@
       <c r="J50" s="8"/>
       <c r="K50" s="8"/>
       <c r="L50" s="8"/>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M50" s="8"/>
+      <c r="N50" s="8"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="8"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
@@ -4753,8 +4873,10 @@
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
       <c r="L51" s="8"/>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M51" s="8"/>
+      <c r="N51" s="8"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="8"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -4767,8 +4889,10 @@
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
       <c r="L52" s="8"/>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M52" s="8"/>
+      <c r="N52" s="8"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="8"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
@@ -4781,8 +4905,10 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
       <c r="L53" s="8"/>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M53" s="8"/>
+      <c r="N53" s="8"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="8"/>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
@@ -4795,8 +4921,10 @@
       <c r="J54" s="8"/>
       <c r="K54" s="8"/>
       <c r="L54" s="8"/>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M54" s="8"/>
+      <c r="N54" s="8"/>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
@@ -4809,8 +4937,10 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
       <c r="L55" s="8"/>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M55" s="8"/>
+      <c r="N55" s="8"/>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="8"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
@@ -4823,8 +4953,10 @@
       <c r="J56" s="8"/>
       <c r="K56" s="8"/>
       <c r="L56" s="8"/>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M56" s="8"/>
+      <c r="N56" s="8"/>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" s="8"/>
       <c r="B57" s="8"/>
       <c r="C57" s="8"/>
@@ -4837,11 +4969,13 @@
       <c r="J57" s="8"/>
       <c r="K57" s="8"/>
       <c r="L57" s="8"/>
+      <c r="M57" s="8"/>
+      <c r="N57" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F57" xr:uid="{00000000-0002-0000-0100-000000000000}">

</xml_diff>

<commit_message>
feat(tabs): wire insight_exclude_categories through; card headers lead with question text
Item 0 + item 2 of DIFFERENCES_TAB_SCOPE.md.

Item 0 — the exclusion lever the JS consumed but nothing could set
(consumed + tested since 2026-08, never written; the alpha_default
class of defect one layer along). Four files: build_config_object
whitelist + TABS_KNOWN_SETTINGS (crosstabs_config.R), proj in
data_layer_writer.R, template registration + regenerated shipped
template. patterns_echo.R already read the key. Default empty, so no
existing report changes until a project sets it.

Item 2 — the Differences card header shows the question text; the
code moves to a hover title. Search still indexes the code and the
pin keeps 'code — title' for crosstab traceability.

Tests: full tabs suite 5092/0 (1 pre-existing skip), diffs_tests.mjs
33/0 incl. new case 29, stat_label_tests.mjs 16/0.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/tabs/templates/Crosstab_Config_Template.xlsx
+++ b/modules/tabs/templates/Crosstab_Config_Template.xlsx
@@ -10,14 +10,15 @@
     <sheet name="Selection" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Base Filters Reference" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Comments" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="AddedSlides" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Population" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ReportText" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="AddedSlides" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Population" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="469">
   <si>
     <t xml:space="preserve">TURAS Crosstab Configuration</t>
   </si>
@@ -61,7 +62,7 @@
     <t xml:space="preserve">structure_file</t>
   </si>
   <si>
-    <t xml:space="preserve">Survey_Structure.xlsx</t>
+    <t xml:space="preserve">Survey_Structure_Template.xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">REQUIRED</t>
@@ -367,6 +368,12 @@
     <t xml:space="preserve">Show mode (most frequent value) for Numeric-type questions (unweighted only).</t>
   </si>
   <si>
+    <t xml:space="preserve">show_numeric_sd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show the Standard Deviation row on Numeric-type questions. Turn off for skewed measures (spend, counts) where the SD exceeds the mean and says less than the bins above it.</t>
+  </si>
+  <si>
     <t xml:space="preserve">show_numeric_outliers</t>
   </si>
   <si>
@@ -742,6 +749,15 @@
     <t xml:space="preserve">Open SAVED copies of the v2 report on a cover page: report title, the Comments sheet's executive summary and background, and the first five Story pins as leading findings. Only affects copies made with Save copy, and only when there is story content to show. FALSE (the default) = saved copies open on the dashboard, as before.</t>
   </si>
   <si>
+    <t xml:space="preserve">html_report_v2_cover_findings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How many Story pins the cover lists as leading findings. Blank = 5. ALL = every pin, however many. When the cover does stop short it says so on the page ("Showing 5 of 12 pinned findings"). Note the exported PowerPoint cover is a single slide and always shows the first 5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whole number of 1 or more, ALL, or leave blank for 5</t>
+  </si>
+  <si>
     <t xml:space="preserve">waves_source</t>
   </si>
   <si>
@@ -832,6 +848,15 @@
     <t xml:space="preserve">Comma-separated question codes, or leave blank</t>
   </si>
   <si>
+    <t xml:space="preserve">insight_exclude_categories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category names (from the Selection sheet's Category column) whose questions the Differences tab and the Group overview KeyShare scan treat as cuts, not outcomes - e.g. imputed or modelled measures a study does not want leading its findings. Case-insensitive; adds to the built-in demographics/corpographics detection. The questions stay in the crosstabs. Blank = built-in detection only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comma-separated category names, or leave blank</t>
+  </si>
+  <si>
     <t xml:space="preserve">READER REPORT (OPTIONAL)</t>
   </si>
   <si>
@@ -1316,6 +1341,24 @@
   </si>
   <si>
     <t xml:space="preserve">Satisfaction is up 5 points, driven by service quality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report Text Overrides (optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leave empty unless this study must word something differently from every other study. Platform wording is edited once, in the Callout Editor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Text key to override for THIS study only, e.g. cards.sig.letters. Find the key by opening a report and pressing ctrl+alt+K, or in the Callout Editor under module 'tabs'. An unknown key stops the report build rather than being ignored.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Replacement wording for this study. Leave blank to use the platform text. Same rules as the editor: inline markup only (strong, em, li, sup...), balanced, no attributes; keep any {placeholders} the key declares.</t>
   </si>
   <si>
     <t xml:space="preserve">Additional Report Slides</t>
@@ -2623,14 +2666,14 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="s">
+      <c r="A49" s="15" t="s">
         <v>116</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C49" s="12" t="s">
-        <v>15</v>
+      <c r="C49" s="16" t="s">
+        <v>4</v>
       </c>
       <c r="D49" s="13" t="s">
         <v>117</v>
@@ -2644,7 +2687,7 @@
         <v>118</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C50" s="12" t="s">
         <v>15</v>
@@ -2661,59 +2704,59 @@
         <v>120</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>121</v>
+        <v>31</v>
       </c>
       <c r="C51" s="12" t="s">
         <v>15</v>
       </c>
       <c r="D51" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="E51" s="14" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="s">
+      <c r="B52" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
+      <c r="C52" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D52" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="B53" s="11" t="s">
+      <c r="A53" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C53" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D53" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E53" s="14" t="s">
-        <v>127</v>
-      </c>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C54" s="12" t="s">
         <v>15</v>
       </c>
       <c r="D54" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="E54" s="14" t="s">
         <v>129</v>
-      </c>
-      <c r="E54" s="14" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="55">
@@ -2721,7 +2764,7 @@
         <v>130</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C55" s="12" t="s">
         <v>15</v>
@@ -2730,7 +2773,7 @@
         <v>131</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="56">
@@ -2738,7 +2781,7 @@
         <v>132</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C56" s="12" t="s">
         <v>15</v>
@@ -2747,15 +2790,15 @@
         <v>133</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B57" s="11" t="n">
-        <v>1</v>
+      <c r="B57" s="11" t="s">
+        <v>127</v>
       </c>
       <c r="C57" s="12" t="s">
         <v>15</v>
@@ -2764,116 +2807,116 @@
         <v>135</v>
       </c>
       <c r="E57" s="14" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="s">
+      <c r="B58" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D58" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
+      <c r="E58" s="14" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="B59" s="11" t="s">
+      <c r="A59" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="B60" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C59" s="16" t="s">
+      <c r="C60" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D59" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="E59" s="14" t="s">
+      <c r="D60" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="E60" s="14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-    </row>
     <row r="61">
-      <c r="A61" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="B61" s="11" t="s">
+      <c r="A61" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B62" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C61" s="12" t="s">
+      <c r="C62" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D61" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="E61" s="14" t="s">
+      <c r="D62" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E62" s="14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9"/>
-    </row>
     <row r="63">
-      <c r="A63" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="B63" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C63" s="16" t="s">
+      <c r="A63" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="9"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C64" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D63" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="E63" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="9" t="s">
+      <c r="D64" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="9"/>
+      <c r="E64" s="14" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="B65" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C65" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D65" s="13" t="s">
+      <c r="A65" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="E65" s="14" t="s">
-        <v>150</v>
-      </c>
+      <c r="B65" s="9"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="9"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B66" s="11" t="n">
         <v>10</v>
@@ -2882,10 +2925,10 @@
         <v>15</v>
       </c>
       <c r="D66" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E66" s="14" t="s">
         <v>152</v>
-      </c>
-      <c r="E66" s="14" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="67">
@@ -2893,7 +2936,7 @@
         <v>153</v>
       </c>
       <c r="B67" s="11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C67" s="12" t="s">
         <v>15</v>
@@ -2902,24 +2945,24 @@
         <v>154</v>
       </c>
       <c r="E67" s="14" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B68" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C68" s="12" t="s">
         <v>15</v>
       </c>
       <c r="D68" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="E68" s="14" t="s">
         <v>157</v>
-      </c>
-      <c r="E68" s="14" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="69">
@@ -2927,7 +2970,7 @@
         <v>158</v>
       </c>
       <c r="B69" s="11" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C69" s="12" t="s">
         <v>15</v>
@@ -2936,7 +2979,7 @@
         <v>159</v>
       </c>
       <c r="E69" s="14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="70">
@@ -2944,7 +2987,7 @@
         <v>160</v>
       </c>
       <c r="B70" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C70" s="12" t="s">
         <v>15</v>
@@ -2953,84 +2996,84 @@
         <v>161</v>
       </c>
       <c r="E70" s="14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="9" t="s">
+      <c r="A71" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="9"/>
+      <c r="B71" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D71" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="E71" s="14" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="B72" s="11" t="s">
+      <c r="A72" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="C72" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D72" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="E72" s="14" t="s">
-        <v>166</v>
-      </c>
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="9"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C73" s="12" t="s">
         <v>15</v>
       </c>
       <c r="D73" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="E73" s="14" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="E73" s="14" t="s">
+      <c r="B74" s="11" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="15" t="s">
+      <c r="C74" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D74" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="B74" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C74" s="16" t="s">
+      <c r="E74" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C75" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D74" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="E74" s="14" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="10" t="s">
+      <c r="D75" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="B75" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="C75" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D75" s="13" t="s">
+      <c r="E75" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="E75" s="14" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="76">
@@ -3038,38 +3081,38 @@
         <v>176</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="C76" s="12" t="s">
         <v>15</v>
       </c>
       <c r="D76" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="E76" s="14" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="E76" s="14" t="s">
+      <c r="B77" s="11" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="15" t="s">
+      <c r="C77" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D77" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="B77" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C77" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D77" s="13" t="s">
+      <c r="E77" s="14" t="s">
         <v>181</v>
-      </c>
-      <c r="E77" s="14" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B78" s="11" t="s">
         <v>35</v>
@@ -3078,15 +3121,15 @@
         <v>4</v>
       </c>
       <c r="D78" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="E78" s="14" t="s">
         <v>184</v>
-      </c>
-      <c r="E78" s="14" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B79" s="11" t="s">
         <v>35</v>
@@ -3095,15 +3138,15 @@
         <v>4</v>
       </c>
       <c r="D79" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="E79" s="14" t="s">
         <v>187</v>
-      </c>
-      <c r="E79" s="14" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B80" s="11" t="s">
         <v>35</v>
@@ -3112,15 +3155,15 @@
         <v>4</v>
       </c>
       <c r="D80" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="E80" s="14" t="s">
         <v>190</v>
-      </c>
-      <c r="E80" s="14" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B81" s="11" t="s">
         <v>35</v>
@@ -3129,15 +3172,15 @@
         <v>4</v>
       </c>
       <c r="D81" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="E81" s="14" t="s">
         <v>193</v>
-      </c>
-      <c r="E81" s="14" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B82" s="11" t="s">
         <v>35</v>
@@ -3146,15 +3189,15 @@
         <v>4</v>
       </c>
       <c r="D82" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="E82" s="14" t="s">
         <v>196</v>
-      </c>
-      <c r="E82" s="14" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B83" s="11" t="s">
         <v>35</v>
@@ -3163,15 +3206,15 @@
         <v>4</v>
       </c>
       <c r="D83" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="E83" s="14" t="s">
         <v>199</v>
-      </c>
-      <c r="E83" s="14" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B84" s="11" t="s">
         <v>35</v>
@@ -3180,15 +3223,15 @@
         <v>4</v>
       </c>
       <c r="D84" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="E84" s="14" t="s">
         <v>202</v>
-      </c>
-      <c r="E84" s="14" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B85" s="11" t="s">
         <v>35</v>
@@ -3197,44 +3240,44 @@
         <v>4</v>
       </c>
       <c r="D85" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="E85" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="E85" s="14" t="s">
+    </row>
+    <row r="86">
+      <c r="A86" s="15" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="10" t="s">
+      <c r="B86" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C86" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D86" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="B86" s="11" t="s">
+      <c r="E86" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="C86" s="12" t="s">
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B87" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="C87" s="12" t="s">
         <v>15</v>
-      </c>
-      <c r="D86" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="E86" s="14" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="B87" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C87" s="16" t="s">
-        <v>4</v>
       </c>
       <c r="D87" s="13" t="s">
         <v>211</v>
       </c>
       <c r="E87" s="14" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="88">
@@ -3251,12 +3294,12 @@
         <v>213</v>
       </c>
       <c r="E88" s="14" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="15" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B89" s="11" t="s">
         <v>35</v>
@@ -3265,10 +3308,10 @@
         <v>4</v>
       </c>
       <c r="D89" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="E89" s="14" t="s">
         <v>216</v>
-      </c>
-      <c r="E89" s="14" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="90">
@@ -3285,41 +3328,41 @@
         <v>218</v>
       </c>
       <c r="E90" s="14" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="15" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="9" t="s">
+      <c r="B91" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C91" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D91" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="B91" s="9"/>
-      <c r="C91" s="9"/>
-      <c r="D91" s="9"/>
-      <c r="E91" s="9"/>
+      <c r="E91" s="14" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="B92" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C92" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D92" s="13" t="s">
+      <c r="A92" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="E92" s="14" t="s">
-        <v>33</v>
-      </c>
+      <c r="B92" s="9"/>
+      <c r="C92" s="9"/>
+      <c r="D92" s="9"/>
+      <c r="E92" s="9"/>
     </row>
     <row r="93">
       <c r="A93" s="15" t="s">
         <v>223</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C93" s="16" t="s">
         <v>4</v>
@@ -3336,7 +3379,7 @@
         <v>225</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C94" s="16" t="s">
         <v>4</v>
@@ -3345,46 +3388,46 @@
         <v>226</v>
       </c>
       <c r="E94" s="14" t="s">
-        <v>227</v>
+        <v>33</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="15" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B95" s="11" t="s">
-        <v>229</v>
+        <v>35</v>
       </c>
       <c r="C95" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E95" s="14" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="15" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>35</v>
+        <v>231</v>
       </c>
       <c r="C96" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D96" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="E96" s="14" t="s">
         <v>233</v>
-      </c>
-      <c r="E96" s="14" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="15" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B97" s="11" t="s">
         <v>35</v>
@@ -3393,10 +3436,10 @@
         <v>4</v>
       </c>
       <c r="D97" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="E97" s="14" t="s">
         <v>236</v>
-      </c>
-      <c r="E97" s="14" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="98">
@@ -3404,7 +3447,7 @@
         <v>237</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C98" s="16" t="s">
         <v>4</v>
@@ -3413,7 +3456,7 @@
         <v>238</v>
       </c>
       <c r="E98" s="14" t="s">
-        <v>33</v>
+        <v>229</v>
       </c>
     </row>
     <row r="99">
@@ -3438,7 +3481,7 @@
         <v>241</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C100" s="16" t="s">
         <v>4</v>
@@ -3447,12 +3490,12 @@
         <v>242</v>
       </c>
       <c r="E100" s="14" t="s">
-        <v>243</v>
+        <v>33</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="15" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B101" s="11" t="s">
         <v>35</v>
@@ -3461,15 +3504,15 @@
         <v>4</v>
       </c>
       <c r="D101" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="E101" s="14" t="s">
         <v>245</v>
-      </c>
-      <c r="E101" s="14" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="15" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B102" s="11" t="s">
         <v>35</v>
@@ -3478,58 +3521,58 @@
         <v>4</v>
       </c>
       <c r="D102" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="E102" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="E102" s="14" t="s">
+    </row>
+    <row r="103">
+      <c r="A103" s="15" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="9" t="s">
+      <c r="B103" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C103" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D103" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="B103" s="9"/>
-      <c r="C103" s="9"/>
-      <c r="D103" s="9"/>
-      <c r="E103" s="9"/>
+      <c r="E103" s="14" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="15" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C104" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E104" s="14" t="s">
-        <v>33</v>
+        <v>254</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="15" t="s">
-        <v>253</v>
-      </c>
-      <c r="B105" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C105" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D105" s="13" t="s">
-        <v>254</v>
-      </c>
-      <c r="E105" s="14" t="s">
-        <v>33</v>
-      </c>
+      <c r="A105" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="B105" s="9"/>
+      <c r="C105" s="9"/>
+      <c r="D105" s="9"/>
+      <c r="E105" s="9"/>
     </row>
     <row r="106">
       <c r="A106" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B106" s="11" t="s">
         <v>39</v>
@@ -3538,7 +3581,7 @@
         <v>4</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E106" s="14" t="s">
         <v>33</v>
@@ -3546,7 +3589,7 @@
     </row>
     <row r="107">
       <c r="A107" s="15" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B107" s="11" t="s">
         <v>39</v>
@@ -3555,7 +3598,7 @@
         <v>4</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E107" s="14" t="s">
         <v>33</v>
@@ -3563,7 +3606,7 @@
     </row>
     <row r="108">
       <c r="A108" s="15" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B108" s="11" t="s">
         <v>39</v>
@@ -3572,58 +3615,58 @@
         <v>4</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E108" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="B109" s="9"/>
-      <c r="C109" s="9"/>
-      <c r="D109" s="9"/>
-      <c r="E109" s="9"/>
+      <c r="A109" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="B109" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C109" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D109" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="E109" s="14" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="15" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C110" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E110" s="14" t="s">
-        <v>264</v>
+        <v>33</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="15" t="s">
-        <v>265</v>
-      </c>
-      <c r="B111" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C111" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D111" s="13" t="s">
+      <c r="A111" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="E111" s="14" t="s">
-        <v>267</v>
-      </c>
+      <c r="B111" s="9"/>
+      <c r="C111" s="9"/>
+      <c r="D111" s="9"/>
+      <c r="E111" s="9"/>
     </row>
     <row r="112">
       <c r="A112" s="15" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B112" s="11" t="s">
         <v>35</v>
@@ -3632,58 +3675,66 @@
         <v>4</v>
       </c>
       <c r="D112" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="E112" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="E112" s="14" t="s">
+    </row>
+    <row r="113">
+      <c r="A113" s="15" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="9" t="s">
+      <c r="B113" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C113" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D113" s="13" t="s">
         <v>271</v>
       </c>
-      <c r="B113" s="9"/>
-      <c r="C113" s="9"/>
-      <c r="D113" s="9"/>
-      <c r="E113" s="9"/>
+      <c r="E113" s="14" t="s">
+        <v>272</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C114" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D114" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E114" s="14" t="s">
-        <v>33</v>
+        <v>275</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="15" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C115" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E115" s="14" t="s">
-        <v>33</v>
+        <v>278</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="9" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B116" s="9"/>
       <c r="C116" s="9"/>
@@ -3692,54 +3743,46 @@
     </row>
     <row r="117">
       <c r="A117" s="15" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C117" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E117" s="14" t="s">
-        <v>206</v>
+        <v>33</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="15" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C118" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D118" s="13" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E118" s="14" t="s">
-        <v>281</v>
+        <v>33</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="15" t="s">
-        <v>282</v>
-      </c>
-      <c r="B119" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C119" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D119" s="13" t="s">
-        <v>283</v>
-      </c>
-      <c r="E119" s="14" t="s">
+      <c r="A119" s="9" t="s">
         <v>284</v>
       </c>
+      <c r="B119" s="9"/>
+      <c r="C119" s="9"/>
+      <c r="D119" s="9"/>
+      <c r="E119" s="9"/>
     </row>
     <row r="120">
       <c r="A120" s="15" t="s">
@@ -3755,7 +3798,7 @@
         <v>286</v>
       </c>
       <c r="E120" s="14" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="121">
@@ -3780,7 +3823,7 @@
         <v>290</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>125</v>
+        <v>35</v>
       </c>
       <c r="C122" s="16" t="s">
         <v>4</v>
@@ -3793,51 +3836,59 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="9" t="s">
+      <c r="A123" s="15" t="s">
         <v>293</v>
       </c>
-      <c r="B123" s="9"/>
-      <c r="C123" s="9"/>
-      <c r="D123" s="9"/>
-      <c r="E123" s="9"/>
+      <c r="B123" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C123" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D123" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="E123" s="14" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C124" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D124" s="13" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E124" s="14" t="s">
-        <v>33</v>
+        <v>297</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="15" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>297</v>
+        <v>127</v>
       </c>
       <c r="C125" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E125" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="9" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B126" s="9"/>
       <c r="C126" s="9"/>
@@ -3846,19 +3897,19 @@
     </row>
     <row r="127">
       <c r="A127" s="15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C127" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D127" s="13" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E127" s="14" t="s">
-        <v>303</v>
+        <v>33</v>
       </c>
     </row>
     <row r="128">
@@ -3866,21 +3917,21 @@
         <v>304</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>35</v>
+        <v>305</v>
       </c>
       <c r="C128" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E128" s="14" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="9" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B129" s="9"/>
       <c r="C129" s="9"/>
@@ -3889,7 +3940,7 @@
     </row>
     <row r="130">
       <c r="A130" s="15" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B130" s="11" t="s">
         <v>35</v>
@@ -3898,66 +3949,58 @@
         <v>4</v>
       </c>
       <c r="D130" s="13" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E130" s="14" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="15" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>311</v>
+        <v>35</v>
       </c>
       <c r="C131" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D131" s="13" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E131" s="14" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="15" t="s">
+      <c r="A132" s="9" t="s">
         <v>314</v>
       </c>
-      <c r="B132" s="11" t="s">
-        <v>315</v>
-      </c>
-      <c r="C132" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D132" s="13" t="s">
-        <v>316</v>
-      </c>
-      <c r="E132" s="14" t="s">
-        <v>317</v>
-      </c>
+      <c r="B132" s="9"/>
+      <c r="C132" s="9"/>
+      <c r="D132" s="9"/>
+      <c r="E132" s="9"/>
     </row>
     <row r="133">
       <c r="A133" s="15" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>319</v>
+        <v>35</v>
       </c>
       <c r="C133" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D133" s="13" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="E133" s="14" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="15" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B134" s="11" t="s">
         <v>319</v>
@@ -3966,44 +4009,95 @@
         <v>4</v>
       </c>
       <c r="D134" s="13" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E134" s="14" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="15" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B135" s="11" t="s">
-        <v>35</v>
+        <v>323</v>
       </c>
       <c r="C135" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D135" s="13" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E135" s="14" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B136" s="11" t="s">
-        <v>35</v>
+        <v>327</v>
       </c>
       <c r="C136" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D136" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="E136" s="14" t="s">
         <v>329</v>
       </c>
-      <c r="E136" s="14" t="s">
+    </row>
+    <row r="137">
+      <c r="A137" s="15" t="s">
         <v>330</v>
+      </c>
+      <c r="B137" s="11" t="s">
+        <v>327</v>
+      </c>
+      <c r="C137" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D137" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="E137" s="14" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="B138" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C138" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D138" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="E138" s="14" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="B139" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C139" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D139" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="E139" s="14" t="s">
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -4017,20 +4111,20 @@
     <mergeCell ref="A32:E32"/>
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A62:E62"/>
-    <mergeCell ref="A64:E64"/>
-    <mergeCell ref="A71:E71"/>
-    <mergeCell ref="A91:E91"/>
-    <mergeCell ref="A103:E103"/>
-    <mergeCell ref="A109:E109"/>
-    <mergeCell ref="A113:E113"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A92:E92"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A111:E111"/>
     <mergeCell ref="A116:E116"/>
-    <mergeCell ref="A123:E123"/>
+    <mergeCell ref="A119:E119"/>
     <mergeCell ref="A126:E126"/>
     <mergeCell ref="A129:E129"/>
+    <mergeCell ref="A132:E132"/>
   </mergeCells>
   <dataValidations count="15">
     <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B27:B27">
@@ -4065,20 +4159,16 @@
       <formula1>1</formula1>
       <formula2>100000</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B57:B57">
+    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B58:B58">
       <formula1>0</formula1>
       <formula2>3</formula2>
-    </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B65:B65">
-      <formula1>1</formula1>
-      <formula2>100</formula2>
     </dataValidation>
     <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B66:B66">
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B67:B67">
-      <formula1>0</formula1>
+    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B67:B67">
+      <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
     <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B68:B68">
@@ -4093,12 +4183,16 @@
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B71:B71">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="51">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="52">
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"xlsx"</xm:f>
@@ -4231,7 +4325,7 @@
           </x14:formula1>
           <xm:sqref>B48:B48</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
@@ -4245,15 +4339,15 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"IQR"</xm:f>
+            <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
           <xm:sqref>B51:B51</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"Y,N"</xm:f>
+            <xm:f>"IQR"</xm:f>
           </x14:formula1>
-          <xm:sqref>B53:B53</xm:sqref>
+          <xm:sqref>B52:B52</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
@@ -4273,29 +4367,29 @@
           </x14:formula1>
           <xm:sqref>B56:B56</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"Y,N"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B57:B57</xm:sqref>
+        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B59:B59</xm:sqref>
+          <xm:sqref>B60:B60</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B61:B61</xm:sqref>
+          <xm:sqref>B62:B62</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"warm,cool,research,teal,red,brand"</xm:f>
           </x14:formula1>
-          <xm:sqref>B76:B76</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>"TRUE,FALSE"</xm:f>
-          </x14:formula1>
-          <xm:sqref>B92:B92</xm:sqref>
+          <xm:sqref>B77:B77</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
@@ -4305,15 +4399,15 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"Not_Specified,Random,Stratified,Cluster,Census,Quota,Online_Panel,Convenience"</xm:f>
+            <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B95:B95</xm:sqref>
+          <xm:sqref>B94:B94</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"TRUE,FALSE"</xm:f>
+            <xm:f>"Not_Specified,Random,Stratified,Cluster,Census,Quota,Online_Panel,Convenience"</xm:f>
           </x14:formula1>
-          <xm:sqref>B98:B98</xm:sqref>
+          <xm:sqref>B96:B96</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
@@ -4325,13 +4419,7 @@
           <x14:formula1>
             <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B104:B104</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>"TRUE,FALSE"</xm:f>
-          </x14:formula1>
-          <xm:sqref>B105:B105</xm:sqref>
+          <xm:sqref>B100:B100</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
@@ -4353,57 +4441,69 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"FALSE,TRUE"</xm:f>
+            <xm:f>"TRUE,FALSE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B114:B114</xm:sqref>
+          <xm:sqref>B109:B109</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"TRUE,FALSE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B110:B110</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"FALSE,TRUE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B115:B115</xm:sqref>
+          <xm:sqref>B117:B117</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>"FALSE,TRUE"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B118:B118</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"Y,N"</xm:f>
           </x14:formula1>
-          <xm:sqref>B122:B122</xm:sqref>
+          <xm:sqref>B125:B125</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"FALSE,TRUE"</xm:f>
           </x14:formula1>
-          <xm:sqref>B124:B124</xm:sqref>
+          <xm:sqref>B127:B127</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"Sonnet 4.6,Opus 4.8"</xm:f>
           </x14:formula1>
-          <xm:sqref>B125:B125</xm:sqref>
+          <xm:sqref>B128:B128</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"hidden,redacted,full"</xm:f>
           </x14:formula1>
-          <xm:sqref>B131:B131</xm:sqref>
+          <xm:sqref>B134:B134</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"allow,safe,block"</xm:f>
           </x14:formula1>
-          <xm:sqref>B132:B132</xm:sqref>
+          <xm:sqref>B135:B135</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"all,noteworthy,must_read,priority"</xm:f>
           </x14:formula1>
-          <xm:sqref>B133:B133</xm:sqref>
+          <xm:sqref>B136:B136</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>"all,noteworthy"</xm:f>
           </x14:formula1>
-          <xm:sqref>B134:B134</xm:sqref>
+          <xm:sqref>B137:B137</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4439,153 +4539,153 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="L4" s="13" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="M4" s="13" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="N4" s="13" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="O4" s="13" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="P4" s="13" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="Q4" s="13" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="R4" s="13" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="S4" s="13" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="F5" s="17" t="n">
         <v>2</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="H5" s="17" t="s">
         <v>35</v>
@@ -4621,18 +4721,18 @@
         <v>35</v>
       </c>
       <c r="S5" s="17" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>35</v>
@@ -4644,7 +4744,7 @@
         <v>35</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>35</v>
@@ -4680,18 +4780,18 @@
         <v>35</v>
       </c>
       <c r="S6" s="17" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>35</v>
@@ -4703,7 +4803,7 @@
         <v>35</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="H7" s="17" t="s">
         <v>35</v>
@@ -4727,10 +4827,10 @@
         <v>35</v>
       </c>
       <c r="O7" s="17" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="P7" s="17" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="Q7" s="17" t="s">
         <v>35</v>
@@ -4739,19 +4839,19 @@
         <v>35</v>
       </c>
       <c r="S7" s="17" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
+        <v>388</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="17" t="s">
         <v>380</v>
       </c>
-      <c r="B8" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>372</v>
-      </c>
       <c r="D8" s="17" t="s">
         <v>35</v>
       </c>
@@ -4762,7 +4862,7 @@
         <v>35</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>35</v>
@@ -4786,19 +4886,19 @@
         <v>35</v>
       </c>
       <c r="O8" s="17" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="P8" s="17" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="Q8" s="17" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="R8" s="17" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="S8" s="17" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
     </row>
     <row r="9">
@@ -5913,122 +6013,122 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
     </row>
   </sheetData>
@@ -6054,48 +6154,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>35</v>
@@ -6106,10 +6206,10 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>35</v>
@@ -6120,10 +6220,10 @@
     </row>
     <row r="7">
       <c r="A7" s="17" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>35</v>
@@ -6134,16 +6234,16 @@
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>35</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
     </row>
     <row r="9">
@@ -6341,6 +6441,131 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
+    <col min="1" max="1" width="40.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="90.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="s">
+        <v>443</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="11"/>
+      <c r="B6" s="11"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
     <col min="1" max="1" width="30.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="70.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
@@ -6348,42 +6573,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>433</v>
+        <v>447</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>434</v>
+        <v>448</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>435</v>
+        <v>449</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>436</v>
+        <v>450</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>437</v>
+        <v>451</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>438</v>
+        <v>452</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>439</v>
+        <v>453</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>440</v>
+        <v>454</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>441</v>
+        <v>455</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>442</v>
+        <v>456</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>1</v>
@@ -6391,10 +6616,10 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>443</v>
+        <v>457</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>444</v>
+        <v>458</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>2</v>
@@ -6516,7 +6741,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -6528,56 +6753,56 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>445</v>
+        <v>459</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>446</v>
+        <v>460</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>447</v>
+        <v>461</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>448</v>
+        <v>462</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>449</v>
+        <v>463</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>450</v>
+        <v>464</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>451</v>
+        <v>465</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>452</v>
+        <v>466</v>
       </c>
       <c r="B5" s="17" t="n">
         <v>27</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>453</v>
+        <v>467</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="s">
-        <v>454</v>
+        <v>468</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>41</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>453</v>
+        <v>467</v>
       </c>
     </row>
     <row r="7">

</xml_diff>